<commit_message>
chore: Add .gitignore to exclude .DS_Store and update annual report data.
</commit_message>
<xml_diff>
--- a/input/children-in-cci/2024-09-22_Data.xlsx
+++ b/input/children-in-cci/2024-09-22_Data.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="3"/>
+    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="CCI_Count" sheetId="1" state="visible" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="48">
   <si>
     <t>District</t>
   </si>
@@ -158,6 +158,9 @@
   </si>
   <si>
     <t>2023-24</t>
+  </si>
+  <si>
+    <t>2024-25</t>
   </si>
   <si>
     <t>average</t>
@@ -175,12 +178,15 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="none"/>
     </fill>
   </fills>
   <borders count="1">
@@ -192,16 +198,20 @@
       <diagonal style="none"/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf fontId="0" fillId="2" borderId="0" numFmtId="9" applyNumberFormat="1" applyFont="0" applyFill="0" applyBorder="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="10" xfId="0" applyNumberFormat="1"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="10" xfId="1" applyNumberFormat="1"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="9" xfId="0" applyNumberFormat="1"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="9" xfId="1" applyNumberFormat="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -589,7 +599,7 @@
     <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr bwMode="auto">
-    <a:xfrm>
+    <a:xfrm rot="0">
       <a:off x="0" y="0"/>
       <a:ext cx="0" cy="0"/>
     </a:xfrm>
@@ -1243,7 +1253,7 @@
           <a:graphicFrameLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
         </xdr:cNvGraphicFramePr>
       </xdr:nvGraphicFramePr>
-      <xdr:xfrm>
+      <xdr:xfrm rot="0">
         <a:off x="0" y="0"/>
         <a:ext cx="0" cy="0"/>
       </xdr:xfrm>
@@ -1770,13 +1780,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="14.25"/>
   <cols>
     <col bestFit="1" customWidth="1" min="1" max="1" width="20.85546875"/>
     <col bestFit="1" customWidth="1" min="2" max="2" width="14.140625"/>
     <col bestFit="1" customWidth="1" min="3" max="3" width="20"/>
     <col bestFit="1" customWidth="1" min="4" max="4" width="17.42578125"/>
-    <col bestFit="1" customWidth="1" min="5" max="5" width="9.140625"/>
+    <col bestFit="1" customWidth="1" min="5" max="5" width="11.375"/>
     <col bestFit="1" customWidth="1" min="6" max="6" width="27.28515625"/>
     <col bestFit="1" customWidth="1" min="7" max="7" width="26.42578125"/>
     <col bestFit="1" customWidth="1" min="8" max="8" width="5.42578125"/>
@@ -1970,7 +1980,7 @@
         <v>14</v>
       </c>
       <c r="B8">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C8">
         <v>1</v>
@@ -1988,7 +1998,7 @@
         <v>2</v>
       </c>
       <c r="H8">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="9">
@@ -2005,7 +2015,7 @@
         <v>2</v>
       </c>
       <c r="E9">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F9">
         <v>0</v>
@@ -2014,7 +2024,7 @@
         <v>3</v>
       </c>
       <c r="H9">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="10">
@@ -2089,10 +2099,10 @@
         <v>0</v>
       </c>
       <c r="G12">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H12">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13">
@@ -2207,7 +2217,7 @@
         <v>7</v>
       </c>
       <c r="C17">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D17">
         <v>2</v>
@@ -2222,7 +2232,7 @@
         <v>1</v>
       </c>
       <c r="H17">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="18">
@@ -2369,7 +2379,7 @@
         <v>0</v>
       </c>
       <c r="E23">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F23">
         <v>0</v>
@@ -2378,7 +2388,7 @@
         <v>1</v>
       </c>
       <c r="H23">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="24">
@@ -2440,7 +2450,7 @@
         <v>33</v>
       </c>
       <c r="B2">
-        <v>2528</v>
+        <v>2164</v>
       </c>
     </row>
     <row r="3">
@@ -2448,7 +2458,7 @@
         <v>34</v>
       </c>
       <c r="B3">
-        <v>1428</v>
+        <v>1447</v>
       </c>
     </row>
     <row r="4">
@@ -2456,7 +2466,7 @@
         <v>35</v>
       </c>
       <c r="B4">
-        <v>192</v>
+        <v>145</v>
       </c>
     </row>
   </sheetData>
@@ -2589,6 +2599,20 @@
         <v>18097</v>
       </c>
     </row>
+    <row r="9" ht="15">
+      <c r="A9" t="s">
+        <v>46</v>
+      </c>
+      <c r="B9">
+        <v>16168</v>
+      </c>
+      <c r="C9">
+        <v>5556</v>
+      </c>
+      <c r="D9">
+        <v>21724</v>
+      </c>
+    </row>
   </sheetData>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>
@@ -2611,7 +2635,7 @@
         <v>36</v>
       </c>
       <c r="B1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="2">
@@ -2670,7 +2694,14 @@
         <v>0.56826199145876555</v>
       </c>
     </row>
-    <row r="9"/>
+    <row r="9">
+      <c r="A9" t="s">
+        <v>46</v>
+      </c>
+      <c r="B9" s="2">
+        <v>0.52880000000000005</v>
+      </c>
+    </row>
   </sheetData>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>
@@ -2696,14 +2727,14 @@
         <v>36</v>
       </c>
       <c r="B1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
         <v>39</v>
       </c>
-      <c r="B2" s="2">
+      <c r="B2" s="3">
         <v>0.42307810567844872</v>
       </c>
     </row>
@@ -2711,7 +2742,7 @@
       <c r="A3" t="s">
         <v>40</v>
       </c>
-      <c r="B3" s="2">
+      <c r="B3" s="3">
         <v>0.42742471126864257</v>
       </c>
     </row>
@@ -2719,7 +2750,7 @@
       <c r="A4" t="s">
         <v>41</v>
       </c>
-      <c r="B4" s="2">
+      <c r="B4" s="3">
         <v>0.39869396131682211</v>
       </c>
     </row>
@@ -2727,7 +2758,7 @@
       <c r="A5" t="s">
         <v>42</v>
       </c>
-      <c r="B5" s="2">
+      <c r="B5" s="3">
         <v>0.37921372133676096</v>
       </c>
     </row>
@@ -2735,7 +2766,7 @@
       <c r="A6" t="s">
         <v>43</v>
       </c>
-      <c r="B6" s="2">
+      <c r="B6" s="3">
         <v>0.35419074400942852</v>
       </c>
     </row>
@@ -2743,7 +2774,7 @@
       <c r="A7" t="s">
         <v>44</v>
       </c>
-      <c r="B7" s="2">
+      <c r="B7" s="3">
         <v>0.37807294431195831</v>
       </c>
     </row>
@@ -2751,8 +2782,16 @@
       <c r="A8" t="s">
         <v>45</v>
       </c>
-      <c r="B8" s="2">
+      <c r="B8" s="3">
         <v>0.42059486459360856</v>
+      </c>
+    </row>
+    <row r="9" ht="15">
+      <c r="A9" t="s">
+        <v>46</v>
+      </c>
+      <c r="B9" s="4">
+        <v>0.4556</v>
       </c>
     </row>
   </sheetData>

</xml_diff>